<commit_message>
feat: activate automatic mutual-exclusion lock (Lay Away Fortaleza 1X suppresses Lay Draw on same match)
</commit_message>
<xml_diff>
--- a/metodos_aprovados/Sinais_Metodos_Aprovados_2026-08-02.xlsx
+++ b/metodos_aprovados/Sinais_Metodos_Aprovados_2026-08-02.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sinais_Aprovados" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U28"/>
+  <dimension ref="A1:U27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1417,32 +1417,32 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>BULGARIA 1</t>
+          <t>DENMARK 1</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Ludogorets x Botev Vratsa</t>
+          <t>Silkeborg x FC Copenhagen</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Ludogorets</t>
+          <t>Silkeborg</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Botev Vratsa</t>
+          <t>FC Copenhagen</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Lay Draw (Fav &lt;= 1.40)</t>
+          <t>Lay Home / DC X2 (Fav Visitante &lt;= 1.65)</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>Match Odds (Draw)</t>
+          <t>Match Odds (Home)</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1451,20 +1451,20 @@
         </is>
       </c>
       <c r="J13" t="n">
-        <v>5.8</v>
+        <v>6.4</v>
       </c>
       <c r="K13" t="n">
-        <v>1.34</v>
+        <v>1.56</v>
       </c>
       <c r="L13" t="n">
-        <v>20.83</v>
+        <v>18.52</v>
       </c>
       <c r="M13" t="n">
         <v>100</v>
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>2x1</t>
+          <t>1x3</t>
         </is>
       </c>
       <c r="O13" t="inlineStr">
@@ -1496,32 +1496,32 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>DENMARK 1</t>
+          <t>ESTONIA 1</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Silkeborg x FC Copenhagen</t>
+          <t>Parnu JK Vaprus x FCI Tallinn</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Silkeborg</t>
+          <t>Parnu JK Vaprus</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>FC Copenhagen</t>
+          <t>FCI Tallinn</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Lay Home / DC X2 (Fav Visitante &lt;= 1.65)</t>
+          <t>Lay Draw (Fav &lt;= 1.40)</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>Match Odds (Home)</t>
+          <t>Match Odds (Draw)</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1530,20 +1530,20 @@
         </is>
       </c>
       <c r="J14" t="n">
-        <v>6.4</v>
+        <v>7.4</v>
       </c>
       <c r="K14" t="n">
-        <v>1.56</v>
+        <v>1.29</v>
       </c>
       <c r="L14" t="n">
-        <v>18.52</v>
+        <v>15.62</v>
       </c>
       <c r="M14" t="n">
         <v>100</v>
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>1x3</t>
+          <t>1x1</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
@@ -1575,22 +1575,22 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>ESTONIA 1</t>
+          <t>PERU 1</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Parnu JK Vaprus x FCI Tallinn</t>
+          <t>Sporting Cristal x Juan Pablo II College</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Parnu JK Vaprus</t>
+          <t>Sporting Cristal</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>FCI Tallinn</t>
+          <t>Juan Pablo II College</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1609,20 +1609,20 @@
         </is>
       </c>
       <c r="J15" t="n">
-        <v>7.4</v>
+        <v>6</v>
       </c>
       <c r="K15" t="n">
-        <v>1.29</v>
+        <v>1.33</v>
       </c>
       <c r="L15" t="n">
-        <v>15.62</v>
+        <v>20</v>
       </c>
       <c r="M15" t="n">
         <v>100</v>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>1x1</t>
+          <t>2x0</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
@@ -1649,37 +1649,37 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>13:30</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>PERU 1</t>
+          <t>CHILE 1</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Sporting Cristal x Juan Pablo II College</t>
+          <t>Deportes Concepcion x Univ Catolica (Chile)</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Sporting Cristal</t>
+          <t>Deportes Concepcion</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Juan Pablo II College</t>
+          <t>Univ Catolica (Chile)</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Lay Draw (Fav &lt;= 1.40)</t>
+          <t>Lay 0x3 Top 3 (Aprovado)</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>Match Odds (Draw)</t>
+          <t>Correct Score (0x3)</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1688,20 +1688,20 @@
         </is>
       </c>
       <c r="J16" t="n">
-        <v>6</v>
+        <v>29</v>
       </c>
       <c r="K16" t="n">
-        <v>1.33</v>
+        <v>0</v>
       </c>
       <c r="L16" t="n">
-        <v>20</v>
+        <v>3.57</v>
       </c>
       <c r="M16" t="n">
         <v>100</v>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>2x0</t>
+          <t>3x0</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
@@ -1733,32 +1733,32 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>CHILE 1</t>
+          <t>CROATIA 1</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Deportes Concepcion x Univ Catolica (Chile)</t>
+          <t>Varazdin x Hajduk Split</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Deportes Concepcion</t>
+          <t>Varazdin</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Univ Catolica (Chile)</t>
+          <t>Hajduk Split</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Lay 0x3 Top 3 (Aprovado)</t>
+          <t>Lay 2x2 Top 3 (Aprovado)</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>Correct Score (0x3)</t>
+          <t>Correct Score (2x2)</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1767,20 +1767,20 @@
         </is>
       </c>
       <c r="J17" t="n">
-        <v>29</v>
+        <v>16.5</v>
       </c>
       <c r="K17" t="n">
         <v>0</v>
       </c>
       <c r="L17" t="n">
-        <v>3.57</v>
+        <v>6.45</v>
       </c>
       <c r="M17" t="n">
         <v>100</v>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>3x0</t>
+          <t>2x1</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
@@ -1807,37 +1807,37 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>13:30</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>CROATIA 1</t>
+          <t>SERBIA 1</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Varazdin x Hajduk Split</t>
+          <t>Zemun x Radnicki Nis</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Varazdin</t>
+          <t>Zemun</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Hajduk Split</t>
+          <t>Radnicki Nis</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Lay 2x2 Top 3 (Aprovado)</t>
+          <t>Lay 0x3 Top 3 (Aprovado)</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>Correct Score (2x2)</t>
+          <t>Correct Score (0x3)</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -1846,20 +1846,20 @@
         </is>
       </c>
       <c r="J18" t="n">
-        <v>16.5</v>
+        <v>29</v>
       </c>
       <c r="K18" t="n">
         <v>0</v>
       </c>
       <c r="L18" t="n">
-        <v>6.45</v>
+        <v>3.57</v>
       </c>
       <c r="M18" t="n">
         <v>100</v>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>2x1</t>
+          <t>0x1</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
@@ -1891,32 +1891,32 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>SERBIA 1</t>
+          <t>ECUADOR 1</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Zemun x Radnicki Nis</t>
+          <t>Independiente (Ecu) x Deportivo Cuenca</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Zemun</t>
+          <t>Independiente (Ecu)</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Radnicki Nis</t>
+          <t>Deportivo Cuenca</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Lay 0x3 Top 3 (Aprovado)</t>
+          <t>Lay Draw (Fav &lt;= 1.40)</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>Correct Score (0x3)</t>
+          <t>Match Odds (Draw)</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -1925,20 +1925,20 @@
         </is>
       </c>
       <c r="J19" t="n">
-        <v>29</v>
+        <v>6.2</v>
       </c>
       <c r="K19" t="n">
-        <v>0</v>
+        <v>1.31</v>
       </c>
       <c r="L19" t="n">
-        <v>3.57</v>
+        <v>19.23</v>
       </c>
       <c r="M19" t="n">
         <v>100</v>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>0x1</t>
+          <t>1x0</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
@@ -1965,27 +1965,27 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>15:15</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>ECUADOR 1</t>
+          <t>BULGARIA 1</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Independiente (Ecu) x Deportivo Cuenca</t>
+          <t>CSKA Sofia x Dunav Ruse</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Independiente (Ecu)</t>
+          <t>CSKA Sofia</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Deportivo Cuenca</t>
+          <t>Dunav Ruse</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -2004,20 +2004,20 @@
         </is>
       </c>
       <c r="J20" t="n">
-        <v>6.2</v>
+        <v>7</v>
       </c>
       <c r="K20" t="n">
-        <v>1.31</v>
+        <v>1.24</v>
       </c>
       <c r="L20" t="n">
-        <v>19.23</v>
+        <v>16.67</v>
       </c>
       <c r="M20" t="n">
         <v>100</v>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>1x0</t>
+          <t>2x1</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
@@ -2044,27 +2044,27 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>15:15</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>BULGARIA 1</t>
+          <t>CROATIA 1</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>CSKA Sofia x Dunav Ruse</t>
+          <t>Rijeka x Rudes</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>CSKA Sofia</t>
+          <t>Rijeka</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Dunav Ruse</t>
+          <t>Rudes</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -2083,13 +2083,13 @@
         </is>
       </c>
       <c r="J21" t="n">
-        <v>7</v>
+        <v>8.4</v>
       </c>
       <c r="K21" t="n">
-        <v>1.24</v>
+        <v>1.21</v>
       </c>
       <c r="L21" t="n">
-        <v>16.67</v>
+        <v>13.51</v>
       </c>
       <c r="M21" t="n">
         <v>100</v>
@@ -2123,37 +2123,37 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>CROATIA 1</t>
+          <t>ARGENTINA 1</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Rijeka x Rudes</t>
+          <t>Newells x Boca Juniors</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Rijeka</t>
+          <t>Newells</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Rudes</t>
+          <t>Boca Juniors</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Lay Draw (Fav &lt;= 1.40)</t>
+          <t>Lay 0x3 Top 3 (Aprovado)</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>Match Odds (Draw)</t>
+          <t>Correct Score (0x3)</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -2162,20 +2162,20 @@
         </is>
       </c>
       <c r="J22" t="n">
-        <v>8.4</v>
+        <v>25</v>
       </c>
       <c r="K22" t="n">
-        <v>1.21</v>
+        <v>0</v>
       </c>
       <c r="L22" t="n">
-        <v>13.51</v>
+        <v>4.17</v>
       </c>
       <c r="M22" t="n">
         <v>100</v>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>2x1</t>
+          <t>2x2</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
@@ -2202,37 +2202,37 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>19:45</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>ARGENTINA 1</t>
+          <t>COLOMBIA 1</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Newells x Boca Juniors</t>
+          <t>America de Cali S.A x Boyaca Chico</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Newells</t>
+          <t>America de Cali S.A</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Boca Juniors</t>
+          <t>Boyaca Chico</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Lay 0x3 Top 3 (Aprovado)</t>
+          <t>Lay Draw (Fav &lt;= 1.40)</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>Correct Score (0x3)</t>
+          <t>Match Odds (Draw)</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -2241,20 +2241,20 @@
         </is>
       </c>
       <c r="J23" t="n">
-        <v>25</v>
+        <v>6.2</v>
       </c>
       <c r="K23" t="n">
-        <v>0</v>
+        <v>1.3</v>
       </c>
       <c r="L23" t="n">
-        <v>4.17</v>
+        <v>19.23</v>
       </c>
       <c r="M23" t="n">
         <v>100</v>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>2x2</t>
+          <t>7x0</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
@@ -2281,37 +2281,37 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>19:45</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>COLOMBIA 1</t>
+          <t>ARGENTINA 1</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>America de Cali S.A x Boyaca Chico</t>
+          <t>Lanus x Instituto</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>America de Cali S.A</t>
+          <t>Lanus</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Boyaca Chico</t>
+          <t>Instituto</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Lay Draw (Fav &lt;= 1.40)</t>
+          <t>Lay Over 4.5 FT (Under Pesado)</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>Match Odds (Draw)</t>
+          <t>Over 4.5 FT</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -2320,20 +2320,20 @@
         </is>
       </c>
       <c r="J24" t="n">
-        <v>6.2</v>
+        <v>19</v>
       </c>
       <c r="K24" t="n">
-        <v>1.3</v>
+        <v>1.48</v>
       </c>
       <c r="L24" t="n">
-        <v>19.23</v>
+        <v>5.56</v>
       </c>
       <c r="M24" t="n">
         <v>100</v>
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>7x0</t>
+          <t>0x1</t>
         </is>
       </c>
       <c r="O24" t="inlineStr">
@@ -2360,37 +2360,29 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>ARGENTINA 1</t>
+          <t>ECUADOR 1</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Lanus x Instituto</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>Lanus</t>
-        </is>
-      </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>Instituto</t>
-        </is>
-      </c>
+          <t>Ind. del Valle x Dep. Cuenca</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr"/>
+      <c r="F25" t="inlineStr"/>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Lay Over 4.5 FT (Under Pesado)</t>
+          <t>Lay Away Fortaleza 1X (Fav &lt;= 1.40 | O25 &gt;= 1.75)</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>Over 4.5 FT</t>
+          <t>Match Odds (Away)</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -2399,37 +2391,43 @@
         </is>
       </c>
       <c r="J25" t="n">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="K25" t="n">
-        <v>1.48</v>
+        <v>1.31</v>
       </c>
       <c r="L25" t="n">
-        <v>5.56</v>
+        <v>8.33</v>
       </c>
       <c r="M25" t="n">
         <v>100</v>
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>0x1</t>
+          <t>1x0</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>PENDENTE</t>
-        </is>
-      </c>
-      <c r="P25" t="inlineStr"/>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="P25" t="n">
+        <v>1</v>
+      </c>
       <c r="Q25" t="inlineStr"/>
-      <c r="R25" t="inlineStr">
-        <is>
-          <t>⏳ PENDENTE</t>
-        </is>
-      </c>
-      <c r="S25" t="inlineStr"/>
-      <c r="T25" t="inlineStr"/>
-      <c r="U25" t="inlineStr"/>
+      <c r="R25" t="inlineStr"/>
+      <c r="S25" t="n">
+        <v>8.039999999999999</v>
+      </c>
+      <c r="T25" t="n">
+        <v>1</v>
+      </c>
+      <c r="U25" t="inlineStr">
+        <is>
+          <t>LIQUIDADO</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -2439,17 +2437,17 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>19:45</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>ECUADOR 1</t>
+          <t>COLOMBIA 1</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Ind. del Valle x Dep. Cuenca</t>
+          <t>America De Cali x Chico</t>
         </is>
       </c>
       <c r="E26" t="inlineStr"/>
@@ -2470,20 +2468,20 @@
         </is>
       </c>
       <c r="J26" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="K26" t="n">
-        <v>1.31</v>
+        <v>1.3</v>
       </c>
       <c r="L26" t="n">
-        <v>8.33</v>
+        <v>7.69</v>
       </c>
       <c r="M26" t="n">
         <v>100</v>
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>1x0</t>
+          <t>7x0</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
@@ -2497,9 +2495,9 @@
       <c r="Q26" t="inlineStr"/>
       <c r="R26" t="inlineStr"/>
       <c r="S26" t="n">
-        <v>8.039999999999999</v>
-      </c>
-      <c r="T26" t="b">
+        <v>7.42</v>
+      </c>
+      <c r="T26" t="n">
         <v>1</v>
       </c>
       <c r="U26" t="inlineStr">
@@ -2516,17 +2514,17 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>19:45</t>
+          <t>13:00</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>COLOMBIA 1</t>
+          <t>BULGARIA 1</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>America De Cali x Chico</t>
+          <t>Ludogorets x Botev Vratsa</t>
         </is>
       </c>
       <c r="E27" t="inlineStr"/>
@@ -2547,20 +2545,20 @@
         </is>
       </c>
       <c r="J27" t="n">
-        <v>14</v>
+        <v>13.5</v>
       </c>
       <c r="K27" t="n">
-        <v>1.3</v>
+        <v>1.34</v>
       </c>
       <c r="L27" t="n">
-        <v>7.69</v>
+        <v>8</v>
       </c>
       <c r="M27" t="n">
         <v>100</v>
       </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>7x0</t>
+          <t>2x1</t>
         </is>
       </c>
       <c r="O27" t="inlineStr">
@@ -2574,89 +2572,12 @@
       <c r="Q27" t="inlineStr"/>
       <c r="R27" t="inlineStr"/>
       <c r="S27" t="n">
-        <v>7.42</v>
-      </c>
-      <c r="T27" t="b">
+        <v>7.72</v>
+      </c>
+      <c r="T27" t="n">
         <v>1</v>
       </c>
       <c r="U27" t="inlineStr">
-        <is>
-          <t>LIQUIDADO</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>2026-08-02</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>13:00</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>BULGARIA 1</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>Ludogorets x Botev Vratsa</t>
-        </is>
-      </c>
-      <c r="E28" t="inlineStr"/>
-      <c r="F28" t="inlineStr"/>
-      <c r="G28" t="inlineStr">
-        <is>
-          <t>Lay Away Fortaleza 1X (Fav &lt;= 1.40 | O25 &gt;= 1.75)</t>
-        </is>
-      </c>
-      <c r="H28" t="inlineStr">
-        <is>
-          <t>Match Odds (Away)</t>
-        </is>
-      </c>
-      <c r="I28" t="inlineStr">
-        <is>
-          <t>LAY</t>
-        </is>
-      </c>
-      <c r="J28" t="n">
-        <v>13.5</v>
-      </c>
-      <c r="K28" t="n">
-        <v>1.34</v>
-      </c>
-      <c r="L28" t="n">
-        <v>8</v>
-      </c>
-      <c r="M28" t="n">
-        <v>100</v>
-      </c>
-      <c r="N28" t="inlineStr">
-        <is>
-          <t>2x1</t>
-        </is>
-      </c>
-      <c r="O28" t="inlineStr">
-        <is>
-          <t>GREEN</t>
-        </is>
-      </c>
-      <c r="P28" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q28" t="inlineStr"/>
-      <c r="R28" t="inlineStr"/>
-      <c r="S28" t="n">
-        <v>7.72</v>
-      </c>
-      <c r="T28" t="b">
-        <v>1</v>
-      </c>
-      <c r="U28" t="inlineStr">
         <is>
           <t>LIQUIDADO</t>
         </is>

</xml_diff>

<commit_message>
feat: integrate Lay 3x0 Top 3 (Aprovado) at 10% B7 Liability across Pages 01, 02, daily automation and Excel sheets
</commit_message>
<xml_diff>
--- a/metodos_aprovados/Sinais_Metodos_Aprovados_2026-08-02.xlsx
+++ b/metodos_aprovados/Sinais_Metodos_Aprovados_2026-08-02.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U27"/>
+  <dimension ref="A1:W30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -534,6 +534,16 @@
           <t>status</t>
         </is>
       </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>PnL_u</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>PnL_R$</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -613,6 +623,8 @@
       <c r="S2" t="inlineStr"/>
       <c r="T2" t="inlineStr"/>
       <c r="U2" t="inlineStr"/>
+      <c r="V2" t="inlineStr"/>
+      <c r="W2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -692,6 +704,8 @@
       <c r="S3" t="inlineStr"/>
       <c r="T3" t="inlineStr"/>
       <c r="U3" t="inlineStr"/>
+      <c r="V3" t="inlineStr"/>
+      <c r="W3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -701,37 +715,37 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>08:35</t>
+          <t>07:30</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>CHINA 1</t>
+          <t>SOUTH KOREA 2</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Liaoning Tieren FC x Shanghai Shenhua</t>
+          <t>Gimpo FC x Gyeongnam</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Liaoning Tieren FC</t>
+          <t>Gimpo FC</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Shanghai Shenhua</t>
+          <t>Gyeongnam</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Lay Home / DC X2 (Fav Visitante &lt;= 1.65)</t>
+          <t>Lay 3x0 Top 3 (Aprovado)</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Match Odds (Home)</t>
+          <t>Correct Score (3x0)</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -740,37 +754,47 @@
         </is>
       </c>
       <c r="J4" t="n">
-        <v>6.4</v>
+        <v>25</v>
       </c>
       <c r="K4" t="n">
-        <v>1.51</v>
+        <v>0</v>
       </c>
       <c r="L4" t="n">
-        <v>18.52</v>
+        <v>8.33</v>
       </c>
       <c r="M4" t="n">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>3x1</t>
+          <t>1x1</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>PENDENTE</t>
-        </is>
-      </c>
-      <c r="P4" t="inlineStr"/>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="P4" t="n">
+        <v>1</v>
+      </c>
       <c r="Q4" t="inlineStr"/>
       <c r="R4" t="inlineStr">
         <is>
-          <t>⏳ PENDENTE</t>
-        </is>
-      </c>
-      <c r="S4" t="inlineStr"/>
+          <t>🟢 GREEN</t>
+        </is>
+      </c>
+      <c r="S4" t="n">
+        <v>8.039999999999999</v>
+      </c>
       <c r="T4" t="inlineStr"/>
       <c r="U4" t="inlineStr"/>
+      <c r="V4" t="n">
+        <v>0.0402</v>
+      </c>
+      <c r="W4" t="n">
+        <v>8.039999999999999</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -780,7 +804,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>09:00</t>
+          <t>08:35</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -790,27 +814,27 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Shenzhen Peng City x Chongqing Tonglianglong</t>
+          <t>Liaoning Tieren FC x Shanghai Shenhua</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Shenzhen Peng City</t>
+          <t>Liaoning Tieren FC</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Chongqing Tonglianglong</t>
+          <t>Shanghai Shenhua</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Lay 2x2 Top 3 (Aprovado)</t>
+          <t>Lay Home / DC X2 (Fav Visitante &lt;= 1.65)</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Correct Score (2x2)</t>
+          <t>Match Odds (Home)</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -819,20 +843,20 @@
         </is>
       </c>
       <c r="J5" t="n">
-        <v>17</v>
+        <v>6.4</v>
       </c>
       <c r="K5" t="n">
-        <v>0</v>
+        <v>1.51</v>
       </c>
       <c r="L5" t="n">
-        <v>6.25</v>
+        <v>18.52</v>
       </c>
       <c r="M5" t="n">
         <v>100</v>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>2x0</t>
+          <t>3x1</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
@@ -850,6 +874,8 @@
       <c r="S5" t="inlineStr"/>
       <c r="T5" t="inlineStr"/>
       <c r="U5" t="inlineStr"/>
+      <c r="V5" t="inlineStr"/>
+      <c r="W5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -864,32 +890,32 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>DENMARK 1</t>
+          <t>CHINA 1</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Midtjylland x AC Horsens</t>
+          <t>Shenzhen Peng City x Chongqing Tonglianglong</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Midtjylland</t>
+          <t>Shenzhen Peng City</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>AC Horsens</t>
+          <t>Chongqing Tonglianglong</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Lay Draw (Fav &lt;= 1.40)</t>
+          <t>Lay 2x2 Top 3 (Aprovado)</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Match Odds (Draw)</t>
+          <t>Correct Score (2x2)</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -898,20 +924,20 @@
         </is>
       </c>
       <c r="J6" t="n">
-        <v>6.2</v>
+        <v>17</v>
       </c>
       <c r="K6" t="n">
-        <v>1.35</v>
+        <v>0</v>
       </c>
       <c r="L6" t="n">
-        <v>19.23</v>
+        <v>6.25</v>
       </c>
       <c r="M6" t="n">
         <v>100</v>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>2x1</t>
+          <t>2x0</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
@@ -929,6 +955,8 @@
       <c r="S6" t="inlineStr"/>
       <c r="T6" t="inlineStr"/>
       <c r="U6" t="inlineStr"/>
+      <c r="V6" t="inlineStr"/>
+      <c r="W6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -938,37 +966,37 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>10:30</t>
+          <t>09:00</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>WALES 1</t>
+          <t>DENMARK 1</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Penybont FC x The New Saints</t>
+          <t>Midtjylland x AC Horsens</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Penybont FC</t>
+          <t>Midtjylland</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>The New Saints</t>
+          <t>AC Horsens</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Lay Home / DC X2 (Fav Visitante &lt;= 1.65)</t>
+          <t>Lay Draw (Fav &lt;= 1.40)</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Match Odds (Home)</t>
+          <t>Match Odds (Draw)</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -977,20 +1005,20 @@
         </is>
       </c>
       <c r="J7" t="n">
-        <v>6.6</v>
+        <v>6.2</v>
       </c>
       <c r="K7" t="n">
-        <v>1.62</v>
+        <v>1.35</v>
       </c>
       <c r="L7" t="n">
-        <v>17.86</v>
+        <v>19.23</v>
       </c>
       <c r="M7" t="n">
         <v>100</v>
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>0x0</t>
+          <t>2x1</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
@@ -1008,6 +1036,8 @@
       <c r="S7" t="inlineStr"/>
       <c r="T7" t="inlineStr"/>
       <c r="U7" t="inlineStr"/>
+      <c r="V7" t="inlineStr"/>
+      <c r="W7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1017,27 +1047,27 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>11:00</t>
+          <t>10:30</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>ICELAND 1</t>
+          <t>WALES 1</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>IA Akranes x Vikingur Reykjavik</t>
+          <t>Penybont FC x The New Saints</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>IA Akranes</t>
+          <t>Penybont FC</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Vikingur Reykjavik</t>
+          <t>The New Saints</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -1056,20 +1086,20 @@
         </is>
       </c>
       <c r="J8" t="n">
-        <v>5.3</v>
+        <v>6.6</v>
       </c>
       <c r="K8" t="n">
-        <v>1.63</v>
+        <v>1.62</v>
       </c>
       <c r="L8" t="n">
-        <v>23.26</v>
+        <v>17.86</v>
       </c>
       <c r="M8" t="n">
         <v>100</v>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>2x2</t>
+          <t>0x0</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
@@ -1087,6 +1117,8 @@
       <c r="S8" t="inlineStr"/>
       <c r="T8" t="inlineStr"/>
       <c r="U8" t="inlineStr"/>
+      <c r="V8" t="inlineStr"/>
+      <c r="W8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1096,37 +1128,37 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>12:00</t>
+          <t>11:00</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>NORWAY 2</t>
+          <t>ICELAND 1</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Kongsvinger x Strommen</t>
+          <t>IA Akranes x Vikingur Reykjavik</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Kongsvinger</t>
+          <t>IA Akranes</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Strommen</t>
+          <t>Vikingur Reykjavik</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Lay Draw (Fav &lt;= 1.40)</t>
+          <t>Lay Home / DC X2 (Fav Visitante &lt;= 1.65)</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Match Odds (Draw)</t>
+          <t>Match Odds (Home)</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -1135,20 +1167,20 @@
         </is>
       </c>
       <c r="J9" t="n">
-        <v>7.2</v>
+        <v>5.3</v>
       </c>
       <c r="K9" t="n">
-        <v>1.32</v>
+        <v>1.63</v>
       </c>
       <c r="L9" t="n">
-        <v>16.13</v>
+        <v>23.26</v>
       </c>
       <c r="M9" t="n">
         <v>100</v>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>1x3</t>
+          <t>2x2</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
@@ -1166,6 +1198,8 @@
       <c r="S9" t="inlineStr"/>
       <c r="T9" t="inlineStr"/>
       <c r="U9" t="inlineStr"/>
+      <c r="V9" t="inlineStr"/>
+      <c r="W9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1185,17 +1219,17 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Odds BK x Asane</t>
+          <t>Kongsvinger x Strommen</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Odds BK</t>
+          <t>Kongsvinger</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Asane</t>
+          <t>Strommen</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -1214,20 +1248,20 @@
         </is>
       </c>
       <c r="J10" t="n">
-        <v>6.6</v>
+        <v>7.2</v>
       </c>
       <c r="K10" t="n">
-        <v>1.35</v>
+        <v>1.32</v>
       </c>
       <c r="L10" t="n">
-        <v>17.86</v>
+        <v>16.13</v>
       </c>
       <c r="M10" t="n">
         <v>100</v>
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>4x1</t>
+          <t>1x3</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
@@ -1245,6 +1279,8 @@
       <c r="S10" t="inlineStr"/>
       <c r="T10" t="inlineStr"/>
       <c r="U10" t="inlineStr"/>
+      <c r="V10" t="inlineStr"/>
+      <c r="W10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1264,27 +1300,27 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Raufoss x Stabaek</t>
+          <t>Odds BK x Asane</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Raufoss</t>
+          <t>Odds BK</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Stabaek</t>
+          <t>Asane</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Lay Home / DC X2 (Fav Visitante &lt;= 1.65)</t>
+          <t>Lay Draw (Fav &lt;= 1.40)</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>Match Odds (Home)</t>
+          <t>Match Odds (Draw)</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -1293,20 +1329,20 @@
         </is>
       </c>
       <c r="J11" t="n">
-        <v>5.4</v>
+        <v>6.6</v>
       </c>
       <c r="K11" t="n">
-        <v>1.63</v>
+        <v>1.35</v>
       </c>
       <c r="L11" t="n">
-        <v>22.73</v>
+        <v>17.86</v>
       </c>
       <c r="M11" t="n">
         <v>100</v>
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>0x2</t>
+          <t>4x1</t>
         </is>
       </c>
       <c r="O11" t="inlineStr">
@@ -1324,6 +1360,8 @@
       <c r="S11" t="inlineStr"/>
       <c r="T11" t="inlineStr"/>
       <c r="U11" t="inlineStr"/>
+      <c r="V11" t="inlineStr"/>
+      <c r="W11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1333,37 +1371,37 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>12:30</t>
+          <t>12:00</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>CZECH 1</t>
+          <t>NORWAY 2</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Bohemians 1905 x Hradec Kralove</t>
+          <t>Raufoss x Stabaek</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Bohemians 1905</t>
+          <t>Raufoss</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Hradec Kralove</t>
+          <t>Stabaek</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Lay 2x2 Top 3 (Aprovado)</t>
+          <t>Lay Home / DC X2 (Fav Visitante &lt;= 1.65)</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>Correct Score (2x2)</t>
+          <t>Match Odds (Home)</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -1372,20 +1410,20 @@
         </is>
       </c>
       <c r="J12" t="n">
-        <v>17.5</v>
+        <v>5.4</v>
       </c>
       <c r="K12" t="n">
-        <v>0</v>
+        <v>1.63</v>
       </c>
       <c r="L12" t="n">
-        <v>6.06</v>
+        <v>22.73</v>
       </c>
       <c r="M12" t="n">
         <v>100</v>
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>0x0</t>
+          <t>0x2</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
@@ -1403,6 +1441,8 @@
       <c r="S12" t="inlineStr"/>
       <c r="T12" t="inlineStr"/>
       <c r="U12" t="inlineStr"/>
+      <c r="V12" t="inlineStr"/>
+      <c r="W12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1412,37 +1452,37 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>12:30</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>DENMARK 1</t>
+          <t>CZECH 1</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Silkeborg x FC Copenhagen</t>
+          <t>Bohemians 1905 x Hradec Kralove</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Silkeborg</t>
+          <t>Bohemians 1905</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>FC Copenhagen</t>
+          <t>Hradec Kralove</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Lay Home / DC X2 (Fav Visitante &lt;= 1.65)</t>
+          <t>Lay 2x2 Top 3 (Aprovado)</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>Match Odds (Home)</t>
+          <t>Correct Score (2x2)</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1451,20 +1491,20 @@
         </is>
       </c>
       <c r="J13" t="n">
-        <v>6.4</v>
+        <v>17.5</v>
       </c>
       <c r="K13" t="n">
-        <v>1.56</v>
+        <v>0</v>
       </c>
       <c r="L13" t="n">
-        <v>18.52</v>
+        <v>6.06</v>
       </c>
       <c r="M13" t="n">
         <v>100</v>
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>1x3</t>
+          <t>0x0</t>
         </is>
       </c>
       <c r="O13" t="inlineStr">
@@ -1482,6 +1522,8 @@
       <c r="S13" t="inlineStr"/>
       <c r="T13" t="inlineStr"/>
       <c r="U13" t="inlineStr"/>
+      <c r="V13" t="inlineStr"/>
+      <c r="W13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1496,32 +1538,32 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>ESTONIA 1</t>
+          <t>DENMARK 1</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Parnu JK Vaprus x FCI Tallinn</t>
+          <t>Silkeborg x FC Copenhagen</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Parnu JK Vaprus</t>
+          <t>Silkeborg</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>FCI Tallinn</t>
+          <t>FC Copenhagen</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Lay Draw (Fav &lt;= 1.40)</t>
+          <t>Lay Home / DC X2 (Fav Visitante &lt;= 1.65)</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>Match Odds (Draw)</t>
+          <t>Match Odds (Home)</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1530,20 +1572,20 @@
         </is>
       </c>
       <c r="J14" t="n">
-        <v>7.4</v>
+        <v>6.4</v>
       </c>
       <c r="K14" t="n">
-        <v>1.29</v>
+        <v>1.56</v>
       </c>
       <c r="L14" t="n">
-        <v>15.62</v>
+        <v>18.52</v>
       </c>
       <c r="M14" t="n">
         <v>100</v>
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>1x1</t>
+          <t>1x3</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
@@ -1561,6 +1603,8 @@
       <c r="S14" t="inlineStr"/>
       <c r="T14" t="inlineStr"/>
       <c r="U14" t="inlineStr"/>
+      <c r="V14" t="inlineStr"/>
+      <c r="W14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1575,22 +1619,22 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>PERU 1</t>
+          <t>ESTONIA 1</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Sporting Cristal x Juan Pablo II College</t>
+          <t>Parnu JK Vaprus x FCI Tallinn</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Sporting Cristal</t>
+          <t>Parnu JK Vaprus</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Juan Pablo II College</t>
+          <t>FCI Tallinn</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1609,20 +1653,20 @@
         </is>
       </c>
       <c r="J15" t="n">
-        <v>6</v>
+        <v>7.4</v>
       </c>
       <c r="K15" t="n">
-        <v>1.33</v>
+        <v>1.29</v>
       </c>
       <c r="L15" t="n">
-        <v>20</v>
+        <v>15.62</v>
       </c>
       <c r="M15" t="n">
         <v>100</v>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>2x0</t>
+          <t>1x1</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
@@ -1640,6 +1684,8 @@
       <c r="S15" t="inlineStr"/>
       <c r="T15" t="inlineStr"/>
       <c r="U15" t="inlineStr"/>
+      <c r="V15" t="inlineStr"/>
+      <c r="W15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1649,37 +1695,37 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>13:30</t>
+          <t>13:00</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>CHILE 1</t>
+          <t>PERU 1</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Deportes Concepcion x Univ Catolica (Chile)</t>
+          <t>Sporting Cristal x Juan Pablo II College</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Deportes Concepcion</t>
+          <t>Sporting Cristal</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Univ Catolica (Chile)</t>
+          <t>Juan Pablo II College</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Lay 0x3 Top 3 (Aprovado)</t>
+          <t>Lay Draw (Fav &lt;= 1.40)</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>Correct Score (0x3)</t>
+          <t>Match Odds (Draw)</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1688,20 +1734,20 @@
         </is>
       </c>
       <c r="J16" t="n">
-        <v>29</v>
+        <v>6</v>
       </c>
       <c r="K16" t="n">
-        <v>0</v>
+        <v>1.33</v>
       </c>
       <c r="L16" t="n">
-        <v>3.57</v>
+        <v>20</v>
       </c>
       <c r="M16" t="n">
         <v>100</v>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>3x0</t>
+          <t>2x0</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
@@ -1719,6 +1765,8 @@
       <c r="S16" t="inlineStr"/>
       <c r="T16" t="inlineStr"/>
       <c r="U16" t="inlineStr"/>
+      <c r="V16" t="inlineStr"/>
+      <c r="W16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1728,37 +1776,29 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>13:30</t>
+          <t>13:00</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>CROATIA 1</t>
+          <t>BULGARIA 1</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Varazdin x Hajduk Split</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>Varazdin</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>Hajduk Split</t>
-        </is>
-      </c>
+          <t>Ludogorets x Botev Vratsa</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr"/>
+      <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Lay 2x2 Top 3 (Aprovado)</t>
+          <t>Lay Away Fortaleza 1X (Fav &lt;= 1.40 | O25 &gt;= 1.75)</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>Correct Score (2x2)</t>
+          <t>Match Odds (Away)</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1767,13 +1807,13 @@
         </is>
       </c>
       <c r="J17" t="n">
-        <v>16.5</v>
+        <v>13.5</v>
       </c>
       <c r="K17" t="n">
-        <v>0</v>
+        <v>1.34</v>
       </c>
       <c r="L17" t="n">
-        <v>6.45</v>
+        <v>8</v>
       </c>
       <c r="M17" t="n">
         <v>100</v>
@@ -1785,19 +1825,27 @@
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>PENDENTE</t>
-        </is>
-      </c>
-      <c r="P17" t="inlineStr"/>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="P17" t="n">
+        <v>1</v>
+      </c>
       <c r="Q17" t="inlineStr"/>
-      <c r="R17" t="inlineStr">
-        <is>
-          <t>⏳ PENDENTE</t>
-        </is>
-      </c>
-      <c r="S17" t="inlineStr"/>
-      <c r="T17" t="inlineStr"/>
-      <c r="U17" t="inlineStr"/>
+      <c r="R17" t="inlineStr"/>
+      <c r="S17" t="n">
+        <v>7.72</v>
+      </c>
+      <c r="T17" t="n">
+        <v>1</v>
+      </c>
+      <c r="U17" t="inlineStr">
+        <is>
+          <t>LIQUIDADO</t>
+        </is>
+      </c>
+      <c r="V17" t="inlineStr"/>
+      <c r="W17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1807,27 +1855,27 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>13:30</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>SERBIA 1</t>
+          <t>CHILE 1</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Zemun x Radnicki Nis</t>
+          <t>Deportes Concepcion x Univ Catolica (Chile)</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Zemun</t>
+          <t>Deportes Concepcion</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Radnicki Nis</t>
+          <t>Univ Catolica (Chile)</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1859,7 +1907,7 @@
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>0x1</t>
+          <t>3x0</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
@@ -1877,6 +1925,8 @@
       <c r="S18" t="inlineStr"/>
       <c r="T18" t="inlineStr"/>
       <c r="U18" t="inlineStr"/>
+      <c r="V18" t="inlineStr"/>
+      <c r="W18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1886,37 +1936,37 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>13:30</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>ECUADOR 1</t>
+          <t>CROATIA 1</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Independiente (Ecu) x Deportivo Cuenca</t>
+          <t>Varazdin x Hajduk Split</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Independiente (Ecu)</t>
+          <t>Varazdin</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Deportivo Cuenca</t>
+          <t>Hajduk Split</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Lay Draw (Fav &lt;= 1.40)</t>
+          <t>Lay 2x2 Top 3 (Aprovado)</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>Match Odds (Draw)</t>
+          <t>Correct Score (2x2)</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -1925,20 +1975,20 @@
         </is>
       </c>
       <c r="J19" t="n">
-        <v>6.2</v>
+        <v>16.5</v>
       </c>
       <c r="K19" t="n">
-        <v>1.31</v>
+        <v>0</v>
       </c>
       <c r="L19" t="n">
-        <v>19.23</v>
+        <v>6.45</v>
       </c>
       <c r="M19" t="n">
         <v>100</v>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>1x0</t>
+          <t>2x1</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
@@ -1956,6 +2006,8 @@
       <c r="S19" t="inlineStr"/>
       <c r="T19" t="inlineStr"/>
       <c r="U19" t="inlineStr"/>
+      <c r="V19" t="inlineStr"/>
+      <c r="W19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1965,37 +2017,37 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>15:15</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>BULGARIA 1</t>
+          <t>SERBIA 1</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>CSKA Sofia x Dunav Ruse</t>
+          <t>Zemun x Radnicki Nis</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>CSKA Sofia</t>
+          <t>Zemun</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Dunav Ruse</t>
+          <t>Radnicki Nis</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Lay Draw (Fav &lt;= 1.40)</t>
+          <t>Lay 0x3 Top 3 (Aprovado)</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>Match Odds (Draw)</t>
+          <t>Correct Score (0x3)</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -2004,20 +2056,20 @@
         </is>
       </c>
       <c r="J20" t="n">
-        <v>7</v>
+        <v>29</v>
       </c>
       <c r="K20" t="n">
-        <v>1.24</v>
+        <v>0</v>
       </c>
       <c r="L20" t="n">
-        <v>16.67</v>
+        <v>3.57</v>
       </c>
       <c r="M20" t="n">
         <v>100</v>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>2x1</t>
+          <t>0x1</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
@@ -2035,6 +2087,8 @@
       <c r="S20" t="inlineStr"/>
       <c r="T20" t="inlineStr"/>
       <c r="U20" t="inlineStr"/>
+      <c r="V20" t="inlineStr"/>
+      <c r="W20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -2044,27 +2098,27 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>CROATIA 1</t>
+          <t>ECUADOR 1</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Rijeka x Rudes</t>
+          <t>Independiente (Ecu) x Deportivo Cuenca</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Rijeka</t>
+          <t>Independiente (Ecu)</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Rudes</t>
+          <t>Deportivo Cuenca</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -2083,20 +2137,20 @@
         </is>
       </c>
       <c r="J21" t="n">
-        <v>8.4</v>
+        <v>6.2</v>
       </c>
       <c r="K21" t="n">
-        <v>1.21</v>
+        <v>1.31</v>
       </c>
       <c r="L21" t="n">
-        <v>13.51</v>
+        <v>19.23</v>
       </c>
       <c r="M21" t="n">
         <v>100</v>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>2x1</t>
+          <t>1x0</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
@@ -2114,6 +2168,8 @@
       <c r="S21" t="inlineStr"/>
       <c r="T21" t="inlineStr"/>
       <c r="U21" t="inlineStr"/>
+      <c r="V21" t="inlineStr"/>
+      <c r="W21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -2123,37 +2179,29 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>ARGENTINA 1</t>
+          <t>ECUADOR 1</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Newells x Boca Juniors</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>Newells</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>Boca Juniors</t>
-        </is>
-      </c>
+          <t>Ind. del Valle x Dep. Cuenca</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr"/>
+      <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Lay 0x3 Top 3 (Aprovado)</t>
+          <t>Lay Away Fortaleza 1X (Fav &lt;= 1.40 | O25 &gt;= 1.75)</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>Correct Score (0x3)</t>
+          <t>Match Odds (Away)</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -2162,37 +2210,45 @@
         </is>
       </c>
       <c r="J22" t="n">
-        <v>25</v>
+        <v>13</v>
       </c>
       <c r="K22" t="n">
-        <v>0</v>
+        <v>1.31</v>
       </c>
       <c r="L22" t="n">
-        <v>4.17</v>
+        <v>8.33</v>
       </c>
       <c r="M22" t="n">
         <v>100</v>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>2x2</t>
+          <t>1x0</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>PENDENTE</t>
-        </is>
-      </c>
-      <c r="P22" t="inlineStr"/>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="P22" t="n">
+        <v>1</v>
+      </c>
       <c r="Q22" t="inlineStr"/>
-      <c r="R22" t="inlineStr">
-        <is>
-          <t>⏳ PENDENTE</t>
-        </is>
-      </c>
-      <c r="S22" t="inlineStr"/>
-      <c r="T22" t="inlineStr"/>
-      <c r="U22" t="inlineStr"/>
+      <c r="R22" t="inlineStr"/>
+      <c r="S22" t="n">
+        <v>8.039999999999999</v>
+      </c>
+      <c r="T22" t="n">
+        <v>1</v>
+      </c>
+      <c r="U22" t="inlineStr">
+        <is>
+          <t>LIQUIDADO</t>
+        </is>
+      </c>
+      <c r="V22" t="inlineStr"/>
+      <c r="W22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -2202,27 +2258,27 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>19:45</t>
+          <t>15:15</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>COLOMBIA 1</t>
+          <t>BULGARIA 1</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>America de Cali S.A x Boyaca Chico</t>
+          <t>CSKA Sofia x Dunav Ruse</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>America de Cali S.A</t>
+          <t>CSKA Sofia</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Boyaca Chico</t>
+          <t>Dunav Ruse</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -2241,20 +2297,20 @@
         </is>
       </c>
       <c r="J23" t="n">
-        <v>6.2</v>
+        <v>7</v>
       </c>
       <c r="K23" t="n">
-        <v>1.3</v>
+        <v>1.24</v>
       </c>
       <c r="L23" t="n">
-        <v>19.23</v>
+        <v>16.67</v>
       </c>
       <c r="M23" t="n">
         <v>100</v>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>7x0</t>
+          <t>2x1</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
@@ -2272,6 +2328,8 @@
       <c r="S23" t="inlineStr"/>
       <c r="T23" t="inlineStr"/>
       <c r="U23" t="inlineStr"/>
+      <c r="V23" t="inlineStr"/>
+      <c r="W23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -2281,37 +2339,37 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>ARGENTINA 1</t>
+          <t>CROATIA 1</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Lanus x Instituto</t>
+          <t>Rijeka x Rudes</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Lanus</t>
+          <t>Rijeka</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Instituto</t>
+          <t>Rudes</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Lay Over 4.5 FT (Under Pesado)</t>
+          <t>Lay Draw (Fav &lt;= 1.40)</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>Over 4.5 FT</t>
+          <t>Match Odds (Draw)</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -2320,20 +2378,20 @@
         </is>
       </c>
       <c r="J24" t="n">
-        <v>19</v>
+        <v>8.4</v>
       </c>
       <c r="K24" t="n">
-        <v>1.48</v>
+        <v>1.21</v>
       </c>
       <c r="L24" t="n">
-        <v>5.56</v>
+        <v>13.51</v>
       </c>
       <c r="M24" t="n">
         <v>100</v>
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>0x1</t>
+          <t>2x1</t>
         </is>
       </c>
       <c r="O24" t="inlineStr">
@@ -2351,6 +2409,8 @@
       <c r="S24" t="inlineStr"/>
       <c r="T24" t="inlineStr"/>
       <c r="U24" t="inlineStr"/>
+      <c r="V24" t="inlineStr"/>
+      <c r="W24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -2360,29 +2420,37 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>ECUADOR 1</t>
+          <t>ARGENTINA 1</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Ind. del Valle x Dep. Cuenca</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr"/>
-      <c r="F25" t="inlineStr"/>
+          <t>Newells x Boca Juniors</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Newells</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Boca Juniors</t>
+        </is>
+      </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Lay Away Fortaleza 1X (Fav &lt;= 1.40 | O25 &gt;= 1.75)</t>
+          <t>Lay 0x3 Top 3 (Aprovado)</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>Match Odds (Away)</t>
+          <t>Correct Score (0x3)</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -2391,43 +2459,39 @@
         </is>
       </c>
       <c r="J25" t="n">
-        <v>13</v>
+        <v>25</v>
       </c>
       <c r="K25" t="n">
-        <v>1.31</v>
+        <v>0</v>
       </c>
       <c r="L25" t="n">
-        <v>8.33</v>
+        <v>4.17</v>
       </c>
       <c r="M25" t="n">
         <v>100</v>
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>1x0</t>
+          <t>2x2</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>GREEN</t>
-        </is>
-      </c>
-      <c r="P25" t="n">
-        <v>1</v>
-      </c>
+          <t>PENDENTE</t>
+        </is>
+      </c>
+      <c r="P25" t="inlineStr"/>
       <c r="Q25" t="inlineStr"/>
-      <c r="R25" t="inlineStr"/>
-      <c r="S25" t="n">
-        <v>8.039999999999999</v>
-      </c>
-      <c r="T25" t="n">
-        <v>1</v>
-      </c>
-      <c r="U25" t="inlineStr">
-        <is>
-          <t>LIQUIDADO</t>
-        </is>
-      </c>
+      <c r="R25" t="inlineStr">
+        <is>
+          <t>⏳ PENDENTE</t>
+        </is>
+      </c>
+      <c r="S25" t="inlineStr"/>
+      <c r="T25" t="inlineStr"/>
+      <c r="U25" t="inlineStr"/>
+      <c r="V25" t="inlineStr"/>
+      <c r="W25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -2437,29 +2501,37 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>19:45</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>COLOMBIA 1</t>
+          <t>BRAZIL CUP</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>America De Cali x Chico</t>
-        </is>
-      </c>
-      <c r="E26" t="inlineStr"/>
-      <c r="F26" t="inlineStr"/>
+          <t>Mirassol x Gremio</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Mirassol</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Gremio</t>
+        </is>
+      </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Lay Away Fortaleza 1X (Fav &lt;= 1.40 | O25 &gt;= 1.75)</t>
+          <t>Lay 3x0 Top 3 (Aprovado)</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>Match Odds (Away)</t>
+          <t>Correct Score (3x0)</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
@@ -2468,20 +2540,20 @@
         </is>
       </c>
       <c r="J26" t="n">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="K26" t="n">
-        <v>1.3</v>
+        <v>0</v>
       </c>
       <c r="L26" t="n">
-        <v>7.69</v>
+        <v>8</v>
       </c>
       <c r="M26" t="n">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>7x0</t>
+          <t>1x1</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
@@ -2493,17 +2565,21 @@
         <v>1</v>
       </c>
       <c r="Q26" t="inlineStr"/>
-      <c r="R26" t="inlineStr"/>
+      <c r="R26" t="inlineStr">
+        <is>
+          <t>🟢 GREEN</t>
+        </is>
+      </c>
       <c r="S26" t="n">
-        <v>7.42</v>
-      </c>
-      <c r="T26" t="n">
-        <v>1</v>
-      </c>
-      <c r="U26" t="inlineStr">
-        <is>
-          <t>LIQUIDADO</t>
-        </is>
+        <v>7.72</v>
+      </c>
+      <c r="T26" t="inlineStr"/>
+      <c r="U26" t="inlineStr"/>
+      <c r="V26" t="n">
+        <v>0.0386</v>
+      </c>
+      <c r="W26" t="n">
+        <v>7.72</v>
       </c>
     </row>
     <row r="27">
@@ -2514,29 +2590,37 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>19:15</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>BULGARIA 1</t>
+          <t>ARGENTINA 1</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Ludogorets x Botev Vratsa</t>
-        </is>
-      </c>
-      <c r="E27" t="inlineStr"/>
-      <c r="F27" t="inlineStr"/>
+          <t>River Plate x Rosario Central</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>River Plate</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Rosario Central</t>
+        </is>
+      </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Lay Away Fortaleza 1X (Fav &lt;= 1.40 | O25 &gt;= 1.75)</t>
+          <t>Lay 3x0 Top 3 (Aprovado)</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>Match Odds (Away)</t>
+          <t>Correct Score (3x0)</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
@@ -2545,20 +2629,20 @@
         </is>
       </c>
       <c r="J27" t="n">
-        <v>13.5</v>
+        <v>23</v>
       </c>
       <c r="K27" t="n">
-        <v>1.34</v>
+        <v>0</v>
       </c>
       <c r="L27" t="n">
-        <v>8</v>
+        <v>9.09</v>
       </c>
       <c r="M27" t="n">
-        <v>100</v>
+        <v>200</v>
       </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>2x1</t>
+          <t>0x1</t>
         </is>
       </c>
       <c r="O27" t="inlineStr">
@@ -2570,18 +2654,263 @@
         <v>1</v>
       </c>
       <c r="Q27" t="inlineStr"/>
-      <c r="R27" t="inlineStr"/>
+      <c r="R27" t="inlineStr">
+        <is>
+          <t>🟢 GREEN</t>
+        </is>
+      </c>
       <c r="S27" t="n">
-        <v>7.72</v>
-      </c>
-      <c r="T27" t="n">
+        <v>8.77</v>
+      </c>
+      <c r="T27" t="inlineStr"/>
+      <c r="U27" t="inlineStr"/>
+      <c r="V27" t="n">
+        <v>0.0439</v>
+      </c>
+      <c r="W27" t="n">
+        <v>8.77</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>19:45</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>COLOMBIA 1</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>America de Cali S.A x Boyaca Chico</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>America de Cali S.A</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Boyaca Chico</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>Lay Draw (Fav &lt;= 1.40)</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>Match Odds (Draw)</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>LAY</t>
+        </is>
+      </c>
+      <c r="J28" t="n">
+        <v>6.2</v>
+      </c>
+      <c r="K28" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="L28" t="n">
+        <v>19.23</v>
+      </c>
+      <c r="M28" t="n">
+        <v>100</v>
+      </c>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>7x0</t>
+        </is>
+      </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>PENDENTE</t>
+        </is>
+      </c>
+      <c r="P28" t="inlineStr"/>
+      <c r="Q28" t="inlineStr"/>
+      <c r="R28" t="inlineStr">
+        <is>
+          <t>⏳ PENDENTE</t>
+        </is>
+      </c>
+      <c r="S28" t="inlineStr"/>
+      <c r="T28" t="inlineStr"/>
+      <c r="U28" t="inlineStr"/>
+      <c r="V28" t="inlineStr"/>
+      <c r="W28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>19:45</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>COLOMBIA 1</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>America De Cali x Chico</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr"/>
+      <c r="F29" t="inlineStr"/>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>Lay Away Fortaleza 1X (Fav &lt;= 1.40 | O25 &gt;= 1.75)</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>Match Odds (Away)</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>LAY</t>
+        </is>
+      </c>
+      <c r="J29" t="n">
+        <v>14</v>
+      </c>
+      <c r="K29" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="L29" t="n">
+        <v>7.69</v>
+      </c>
+      <c r="M29" t="n">
+        <v>100</v>
+      </c>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>7x0</t>
+        </is>
+      </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="P29" t="n">
         <v>1</v>
       </c>
-      <c r="U27" t="inlineStr">
+      <c r="Q29" t="inlineStr"/>
+      <c r="R29" t="inlineStr"/>
+      <c r="S29" t="n">
+        <v>7.42</v>
+      </c>
+      <c r="T29" t="n">
+        <v>1</v>
+      </c>
+      <c r="U29" t="inlineStr">
         <is>
           <t>LIQUIDADO</t>
         </is>
       </c>
+      <c r="V29" t="inlineStr"/>
+      <c r="W29" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>21:30</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>ARGENTINA 1</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Lanus x Instituto</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Lanus</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Instituto</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>Lay Over 4.5 FT (Under Pesado)</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>Over 4.5 FT</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>LAY</t>
+        </is>
+      </c>
+      <c r="J30" t="n">
+        <v>19</v>
+      </c>
+      <c r="K30" t="n">
+        <v>1.48</v>
+      </c>
+      <c r="L30" t="n">
+        <v>5.56</v>
+      </c>
+      <c r="M30" t="n">
+        <v>100</v>
+      </c>
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>0x1</t>
+        </is>
+      </c>
+      <c r="O30" t="inlineStr">
+        <is>
+          <t>PENDENTE</t>
+        </is>
+      </c>
+      <c r="P30" t="inlineStr"/>
+      <c r="Q30" t="inlineStr"/>
+      <c r="R30" t="inlineStr">
+        <is>
+          <t>⏳ PENDENTE</t>
+        </is>
+      </c>
+      <c r="S30" t="inlineStr"/>
+      <c r="T30" t="inlineStr"/>
+      <c r="U30" t="inlineStr"/>
+      <c r="V30" t="inlineStr"/>
+      <c r="W30" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>